<commit_message>
Fix rate formula showing tariffs 100x too high in summary exports
Rate cells (E/K) in summary templates use the 0.00% number format, which
already multiplies by 100 on display. Commit 942ebf2 changed the template
formula to premium/sum*100, so a 2% tariff rendered as 200%.

Drop *100 from all four summary templates and from the fallback
_create_rate_formula, and add an invariant test that fails whenever a
rate cell with a percent format carries a *100 formula (templates,
fallback formula and every rate row of generated exports).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/client_summary_template.xlsx
+++ b/templates/client_summary_template.xlsx
@@ -1068,7 +1068,7 @@
       <x:c r="C10" s="35" t="n"/>
       <x:c r="D10" s="18" t="n"/>
       <x:c r="E10" s="27" t="str">
-        <x:f>IF(AND(C10&lt;&gt;0,F10&lt;&gt;0),F10/C10*100,"")</x:f>
+        <x:f>IF(AND(C10&lt;&gt;0,F10&lt;&gt;0),F10/C10,"")</x:f>
       </x:c>
       <x:c r="F10" s="28" t="n"/>
       <x:c r="G10" s="29" t="n"/>
@@ -1079,7 +1079,7 @@
       </x:c>
       <x:c r="J10" s="18" t="n"/>
       <x:c r="K10" s="30" t="str">
-        <x:f>IF(AND(C10&lt;&gt;0,L10&lt;&gt;0),L10/C10*100,"")</x:f>
+        <x:f>IF(AND(C10&lt;&gt;0,L10&lt;&gt;0),L10/C10,"")</x:f>
       </x:c>
       <x:c r="L10" s="31" t="n"/>
       <x:c r="M10" s="32" t="n"/>

</xml_diff>